<commit_message>
feat: output an excel files with formulas for calculated cells
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/output_example.xlsx
+++ b/data/examples/output_example.xlsx
@@ -444,67 +444,67 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>Mar.30</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>4.06</t>
+          <t>Apr.06</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>Apr.13</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>Apr.20</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>Apr.27</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>5.04</t>
+          <t>May.04</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>5.11</t>
+          <t>May.11</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>5.18</t>
+          <t>May.18</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>May.25</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>6.01</t>
+          <t>Jun.01</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>6.08</t>
+          <t>Jun.08</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>6.15</t>
+          <t>Jun.15</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>6.22</t>
+          <t>Jun.22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fractional FTEs, refactor: renamed columns
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/output_example.xlsx
+++ b/data/examples/output_example.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1109,320 +1109,56 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Weekly Allocation</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Engineers capacity</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Managers capacity</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Engineers absence</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Managers absence</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Weekly Allocation</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="G18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="H18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="I18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="K18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="L18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="M18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="N18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="O18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="P18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="R18" t="n">
         <v>4.3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: conditional formatting formulas
</commit_message>
<xml_diff>
--- a/data/examples/output_example.xlsx
+++ b/data/examples/output_example.xlsx
@@ -52,6 +52,83 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00548235"/>
+          <bgColor rgb="00548235"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00B4C6E7"/>
+          <bgColor rgb="00B4C6E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D2E9"/>
+          <bgColor rgb="00D9D2E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+          <bgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+          <bgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8CBAD"/>
+          <bgColor rgb="00F8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -522,7 +599,9 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>65</v>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>5</v>
@@ -573,7 +652,9 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>2.6</v>
+      </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>0.2</v>
@@ -624,7 +705,9 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>62.4</v>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>4.8</v>
@@ -675,7 +758,9 @@
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>26</v>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>2</v>
@@ -726,7 +811,9 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>3.9</v>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>0.3</v>
@@ -777,7 +864,9 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>22.1</v>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>1.7</v>
@@ -1245,6 +1334,42 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F8:F12">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>F8=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G14:S14">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
+      <formula>G14=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:S14">
+    <cfRule type="expression" priority="3" dxfId="1" stopIfTrue="0">
+      <formula>$A2="Self-Service ML EV Range - Phase 1"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2" stopIfTrue="0">
+      <formula>$A2="Quality improvements through ML/AI experimentation"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3" stopIfTrue="0">
+      <formula>$A2="Maintenance &amp; Release"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4" stopIfTrue="0">
+      <formula>$A2="Security &amp; Compliance"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="5" stopIfTrue="0">
+      <formula>$A2="Customer Support"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="6" stopIfTrue="0">
+      <formula>$A2="Critical Technical Debt"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="7" stopIfTrue="0">
+      <formula>$A2="Critical Product Debt"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="8" stopIfTrue="0">
+      <formula>$A2="Critical Customer Commitments"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>